<commit_message>
NPB自動更新(1軍): 2026-08-28 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-08-28.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-08-28.xlsx
@@ -103104,7 +103104,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3回に勝ち越し3ラン、5回に2ランと2本塁打5打点の大活躍で勝利に貢献。</t>
+          <t>3回に勝ち越し3ラン、5回にも2ランを放ち、計5打点の大活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -103119,17 +103119,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>牧 秀悟</t>
+          <t>髙橋 宏斗</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>中日</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>8回裏、同点に追いついた直後に勝ち越しのタイムリー二塁打を放ち、チームを勝利に導いた。</t>
+          <t>7回を投げ1失点8奪三振の快投で、相手打線を完全に支配した。</t>
         </is>
       </c>
     </row>
@@ -103144,17 +103144,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>髙橋 宏斗</t>
+          <t>度会 隆輝</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7回を投げ1失点8奪三振の快投で試合を支配したが、救援陣が打たれ勝利を逃した。</t>
+          <t>8回裏2死満塁から同点タイムリーを放ち、チームの逆転劇の口火を切った。</t>
         </is>
       </c>
     </row>
@@ -103169,17 +103169,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>奥川 恭伸</t>
+          <t>牧 秀悟</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8回1失点5奪三振の好投で試合を作り、さらに自らタイムリーも放ち投打で勝利に貢献。</t>
+          <t>8回裏に勝ち越しのタイムリーツーベースを放ち、チームの逆転勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -103204,7 +103204,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回を無失点に抑える好投で試合を作り、チームの勝利に大きく貢献した。</t>
+          <t>7回を投げ被安打4、無失点の好投で、相手打線を完璧に抑え込んだ。</t>
         </is>
       </c>
     </row>
@@ -103229,7 +103229,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1回裏に先制3ランを放ち、さらにタイムリーで計5打点と打線を牽引した。</t>
+          <t>1回裏に先制3ランホームランを放ち、さらに3回にもタイムリーで計5打点。</t>
         </is>
       </c>
     </row>

</xml_diff>